<commit_message>
Update guests.xlsx über Config-Seite
</commit_message>
<xml_diff>
--- a/guests.xlsx
+++ b/guests.xlsx
@@ -484,7 +484,7 @@
         <v>Hoffmann</v>
       </c>
       <c r="C8" t="str">
-        <v>Tisch 2 - Lavendel</v>
+        <v>moin</v>
       </c>
     </row>
     <row r="9">
@@ -506,7 +506,7 @@
         <v>Wagner</v>
       </c>
       <c r="C10" t="str">
-        <v>Tisch 3 - Pfingstrose</v>
+        <v>moin</v>
       </c>
     </row>
     <row r="11">
@@ -550,7 +550,7 @@
         <v>Schulz</v>
       </c>
       <c r="C14" t="str">
-        <v>Tisch 5 - Kamille</v>
+        <v>Tisch 2 - Lavendel</v>
       </c>
     </row>
     <row r="15">
@@ -561,7 +561,7 @@
         <v>Schulz</v>
       </c>
       <c r="C15" t="str">
-        <v>Tisch 5 - Kamille</v>
+        <v>moin</v>
       </c>
     </row>
     <row r="16">
@@ -594,7 +594,7 @@
         <v>Zimmermann</v>
       </c>
       <c r="C18" t="str">
-        <v>Tisch 6 - Vergissmeinnicht</v>
+        <v>moin</v>
       </c>
     </row>
     <row r="19">

</xml_diff>